<commit_message>
Final project AT04, Khang Nguyen, updated
</commit_message>
<xml_diff>
--- a/data/test_cases/update_profile.xlsx
+++ b/data/test_cases/update_profile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nguyentuanminhkhang/Documents/Python/PlaywrightPython/khang0912_final_project/final-project-at04-khangnguyen/data/test_cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA9A560-2448-7C4A-A8C1-83A82BD89FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D927C14F-8220-3B4C-9A08-A5EF3C4F218F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="multiple_fields_ui" sheetId="4" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="87">
   <si>
     <t>case_name</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>{{random_generated_email}}</t>
+  </si>
+  <si>
+    <t>Verify that user can reload My Profile page and the page still opens normally</t>
   </si>
 </sst>
 </file>
@@ -359,7 +362,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -411,6 +414,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -714,11 +721,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986DE7F0-57DF-274B-957F-4BE5AC773E6B}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="78.1640625" style="2" customWidth="1"/>
-    <col min="2" max="7" width="20.5" customWidth="1"/>
+    <col min="2" max="2" width="20.5" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" customWidth="1"/>
+    <col min="4" max="7" width="20.5" customWidth="1"/>
     <col min="8" max="9" width="21.5" customWidth="1"/>
     <col min="10" max="10" width="19.1640625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
@@ -779,65 +788,54 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6"/>
+        <v>86</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="5" t="b">
-        <v>1</v>
-      </c>
+      <c r="H5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6"/>
     </row>
     <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="4"/>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6"/>
+        <v>82</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="4"/>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
       <c r="H7" s="5" t="b">
         <v>1</v>
       </c>
@@ -845,62 +843,61 @@
     </row>
     <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="2"/>
+        <v>56</v>
+      </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="5" t="b">
-        <v>1</v>
-      </c>
+      <c r="H8" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6"/>
     </row>
     <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="H9" s="6"/>
+      <c r="I9" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="5" t="b">
-        <v>1</v>
-      </c>
+      <c r="H10" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -913,75 +910,82 @@
     </row>
     <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="D12" s="2"/>
-      <c r="E12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" t="s">
-        <v>53</v>
-      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="5" t="b">
+      <c r="I12" s="5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="E13" t="s">
+        <v>52</v>
+      </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="G13" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
-      <c r="K13" s="5" t="b">
+      <c r="J13" s="5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="K14" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="C15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="6"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="6"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="I15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
@@ -1011,6 +1015,8 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
@@ -1051,6 +1057,14 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1065,7 +1079,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="D6" numberStoredAsText="1"/>
+    <ignoredError sqref="D7 D15" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1084,26 +1098,26 @@
     <col min="7" max="7" width="44.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" s="20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="20" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>